<commit_message>
feat: add T view for 2026
</commit_message>
<xml_diff>
--- a/data/premissas_valuation.xlsx
+++ b/data/premissas_valuation.xlsx
@@ -37,7 +37,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -48,6 +48,9 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
       </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -72,9 +75,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -86,16 +92,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -463,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:S7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -481,6 +487,10 @@
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -520,280 +530,327 @@
       <c r="J1" s="1" t="n">
         <v>2025</v>
       </c>
-      <c r="K1" s="1" t="n">
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>1T-2026</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>2T-2026</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>3T-2026</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>4T-2026</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="n">
         <v>2026</v>
       </c>
-      <c r="L1" s="1" t="n">
+      <c r="P1" s="1" t="n">
         <v>2027</v>
       </c>
-      <c r="M1" s="1" t="n">
+      <c r="Q1" s="1" t="n">
         <v>2028</v>
       </c>
-      <c r="N1" s="1" t="n">
+      <c r="R1" s="1" t="n">
         <v>2029</v>
       </c>
-      <c r="O1" s="1" t="n">
+      <c r="S1" s="1" t="n">
         <v>2030</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>IPCA</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>% a.a. (variação acumulada no ano)</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>IBGE/SIDRA (histórico) + Focus/BCB (projeção)</t>
         </is>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="D2" s="6" t="n">
         <v>4.31</v>
       </c>
-      <c r="E2" s="5" t="n">
+      <c r="E2" s="6" t="n">
         <v>4.52</v>
       </c>
-      <c r="F2" s="5" t="n">
+      <c r="F2" s="6" t="n">
         <v>10.06</v>
       </c>
-      <c r="G2" s="5" t="n">
+      <c r="G2" s="6" t="n">
         <v>5.79</v>
       </c>
-      <c r="H2" s="5" t="n">
+      <c r="H2" s="6" t="n">
         <v>4.62</v>
       </c>
-      <c r="I2" s="5" t="n">
+      <c r="I2" s="6" t="n">
         <v>4.83</v>
       </c>
-      <c r="J2" s="5" t="n">
+      <c r="J2" s="6" t="n">
         <v>4.26</v>
       </c>
       <c r="K2" s="6" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="L2" s="6" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="O2" s="7" t="n">
         <v>5.3001</v>
       </c>
-      <c r="L2" s="6" t="n">
+      <c r="P2" s="7" t="n">
         <v>4.1818</v>
       </c>
-      <c r="M2" s="6" t="n">
+      <c r="Q2" s="7" t="n">
         <v>3.7</v>
       </c>
-      <c r="N2" s="6" t="n">
+      <c r="R2" s="7" t="n">
         <v>3.5</v>
       </c>
-      <c r="O2" s="6" t="n">
+      <c r="S2" s="7" t="n">
         <v>3.5</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Selic</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>% a.a. (taxa básica de juros)</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>BCB SGS 432 (histórico) + Focus/BCB (projeção)</t>
         </is>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="D3" s="7" t="n">
         <v>4.5</v>
       </c>
-      <c r="E3" s="5" t="n">
+      <c r="E3" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F3" s="5" t="n">
+      <c r="F3" s="7" t="n">
         <v>9.25</v>
       </c>
-      <c r="G3" s="5" t="n">
+      <c r="G3" s="7" t="n">
         <v>13.75</v>
       </c>
-      <c r="H3" s="5" t="n">
+      <c r="H3" s="7" t="n">
         <v>11.75</v>
       </c>
-      <c r="I3" s="5" t="n">
-        <v>12.25</v>
-      </c>
-      <c r="J3" s="5" t="n">
+      <c r="I3" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="J3" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="K3" s="6" t="n">
+      <c r="O3" s="7" t="n">
         <v>14</v>
       </c>
-      <c r="L3" s="6" t="n">
+      <c r="P3" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="M3" s="6" t="n">
+      <c r="Q3" s="7" t="n">
         <v>10.5</v>
       </c>
-      <c r="N3" s="6" t="n">
+      <c r="R3" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="O3" s="6" t="n">
+      <c r="S3" s="7" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>PIB</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>% a.a. (variação do PIB no ano)</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>IBGE/SIDRA (histórico) + Focus/BCB (projeção)</t>
         </is>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D4" s="6" t="n">
         <v>1.3</v>
       </c>
-      <c r="E4" s="5" t="n">
+      <c r="E4" s="6" t="n">
         <v>-3.3</v>
       </c>
-      <c r="F4" s="5" t="n">
+      <c r="F4" s="6" t="n">
         <v>4.8</v>
       </c>
-      <c r="G4" s="5" t="n">
+      <c r="G4" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H4" s="5" t="n">
+      <c r="H4" s="6" t="n">
         <v>3.2</v>
       </c>
-      <c r="I4" s="6" t="n">
+      <c r="I4" s="7" t="n">
         <v>3.4921</v>
       </c>
-      <c r="J4" s="6" t="n">
+      <c r="J4" s="7" t="n">
         <v>2.275</v>
       </c>
-      <c r="K4" s="6" t="n">
+      <c r="O4" s="7" t="n">
         <v>1.9859</v>
       </c>
-      <c r="L4" s="6" t="n">
+      <c r="P4" s="7" t="n">
         <v>1.6895</v>
       </c>
-      <c r="M4" s="6" t="n">
+      <c r="Q4" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="N4" s="6" t="n">
+      <c r="R4" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="O4" s="6" t="n">
+      <c r="S4" s="7" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Ouro</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>USD/onça troy</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>Yahoo Finance (GC=F)</t>
         </is>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D5" s="8" t="n">
         <v>1519.5</v>
       </c>
-      <c r="E5" s="7" t="n">
+      <c r="E5" s="8" t="n">
         <v>1893.1</v>
       </c>
-      <c r="F5" s="7" t="n">
+      <c r="F5" s="8" t="n">
         <v>1827.5</v>
       </c>
-      <c r="G5" s="7" t="n">
+      <c r="G5" s="8" t="n">
         <v>1819.7</v>
       </c>
-      <c r="H5" s="7" t="n">
+      <c r="H5" s="8" t="n">
         <v>2062.4</v>
       </c>
-      <c r="I5" s="7" t="n">
+      <c r="I5" s="8" t="n">
         <v>2629.2</v>
       </c>
-      <c r="J5" s="7" t="n">
+      <c r="J5" s="8" t="n">
         <v>4325.6</v>
       </c>
-      <c r="K5" s="7" t="n">
-        <v>4109.8</v>
+      <c r="K5" s="8" t="n">
+        <v>4647.6</v>
+      </c>
+      <c r="L5" s="8" t="n">
+        <v>4022.9</v>
+      </c>
+      <c r="M5" s="8" t="n">
+        <v>4128.9</v>
+      </c>
+      <c r="O5" s="8" t="n">
+        <v>4128.9</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Prata</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>USD/onça troy</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Yahoo Finance (SI=F)</t>
         </is>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D6" s="8" t="n">
         <v>17.83</v>
       </c>
-      <c r="E6" s="7" t="n">
+      <c r="E6" s="8" t="n">
         <v>26.33</v>
       </c>
-      <c r="F6" s="7" t="n">
+      <c r="F6" s="8" t="n">
         <v>23.33</v>
       </c>
-      <c r="G6" s="7" t="n">
+      <c r="G6" s="8" t="n">
         <v>23.86</v>
       </c>
-      <c r="H6" s="7" t="n">
+      <c r="H6" s="8" t="n">
         <v>23.85</v>
       </c>
-      <c r="I6" s="7" t="n">
+      <c r="I6" s="8" t="n">
         <v>28.94</v>
       </c>
-      <c r="J6" s="7" t="n">
+      <c r="J6" s="8" t="n">
         <v>70.13</v>
       </c>
-      <c r="K6" s="7" t="n">
-        <v>60.03</v>
+      <c r="K6" s="8" t="n">
+        <v>74.69</v>
+      </c>
+      <c r="L6" s="8" t="n">
+        <v>59.48</v>
+      </c>
+      <c r="M6" s="8" t="n">
+        <v>60.3</v>
+      </c>
+      <c r="O6" s="8" t="n">
+        <v>60.3</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>USD/BRL</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>BRL</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>BCB SGS 1 (PTAX)</t>
         </is>
       </c>
-      <c r="K7" s="8" t="n">
+      <c r="M7" s="9" t="n">
+        <v>5.1088</v>
+      </c>
+      <c r="O7" s="9" t="n">
         <v>5.1088</v>
       </c>
     </row>

</xml_diff>